<commit_message>
docs: update feature planning spreadsheet
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SAT_Feature_Planning.xlsx
+++ b/docs/SAT_Feature_Planning.xlsx
@@ -188,7 +188,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -238,11 +238,88 @@
         <color rgb="00AAAAAA"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00888888"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00888888"/>
+      </right>
+      <top style="medium">
+        <color rgb="00888888"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00888888"/>
+      </right>
+      <top style="medium">
+        <color rgb="00888888"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00888888"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -331,6 +408,9 @@
     <xf numFmtId="0" fontId="10" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -740,18 +820,21 @@
 20</t>
         </is>
       </c>
+      <c r="C7" s="32" t="n"/>
       <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Stories Done (Jira)
 4</t>
         </is>
       </c>
+      <c r="E7" s="32" t="n"/>
       <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Stories In Progress
 4</t>
         </is>
       </c>
+      <c r="G7" s="32" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1"/>
     <row r="10" ht="44" customHeight="1">
@@ -761,18 +844,21 @@
 12</t>
         </is>
       </c>
+      <c r="C10" s="32" t="n"/>
       <c r="D10" s="5" t="inlineStr">
         <is>
           <t>Features with Code
 9</t>
         </is>
       </c>
+      <c r="E10" s="32" t="n"/>
       <c r="F10" s="7" t="inlineStr">
         <is>
           <t>Open Issues
 18</t>
         </is>
       </c>
+      <c r="G10" s="32" t="n"/>
     </row>
     <row r="13" ht="44" customHeight="1">
       <c r="B13" s="8" t="inlineStr">
@@ -781,12 +867,14 @@
 4 / 6 needed</t>
         </is>
       </c>
+      <c r="C13" s="32" t="n"/>
       <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Sprint 3 Ready
 3 services</t>
         </is>
       </c>
+      <c r="E13" s="32" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="9" t="inlineStr">
@@ -797,6 +885,7 @@
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="10" t="n"/>
+      <c r="C17" s="33" t="n"/>
       <c r="D17" s="11" t="inlineStr">
         <is>
           <t>Done — Jira resolved + code found</t>
@@ -805,6 +894,7 @@
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="12" t="n"/>
+      <c r="C18" s="33" t="n"/>
       <c r="D18" s="11" t="inlineStr">
         <is>
           <t>In Progress — partial / POC / unverified</t>
@@ -813,6 +903,7 @@
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="13" t="n"/>
+      <c r="C19" s="33" t="n"/>
       <c r="D19" s="11" t="inlineStr">
         <is>
           <t>Not Started — no code, no ticket</t>
@@ -832,11 +923,15 @@
           <t>1. Feature Registry</t>
         </is>
       </c>
+      <c r="C22" s="33" t="n"/>
       <c r="D22" s="15" t="inlineStr">
         <is>
           <t>All 20 stories — status, owner, code location, contract, flag, FVD</t>
         </is>
       </c>
+      <c r="E22" s="34" t="n"/>
+      <c r="F22" s="34" t="n"/>
+      <c r="G22" s="33" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="14" t="inlineStr">
@@ -844,11 +939,15 @@
           <t>2. Integration Plan</t>
         </is>
       </c>
+      <c r="C23" s="33" t="n"/>
       <c r="D23" s="15" t="inlineStr">
         <is>
           <t>Ordered integration queue — 13 items, prerequisites, sprint, blockers</t>
         </is>
       </c>
+      <c r="E23" s="34" t="n"/>
+      <c r="F23" s="34" t="n"/>
+      <c r="G23" s="33" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="14" t="inlineStr">
@@ -856,11 +955,15 @@
           <t>3. Open Issues</t>
         </is>
       </c>
+      <c r="C24" s="33" t="n"/>
       <c r="D24" s="15" t="inlineStr">
         <is>
           <t>18 open issues — severity, owner, status</t>
         </is>
       </c>
+      <c r="E24" s="34" t="n"/>
+      <c r="F24" s="34" t="n"/>
+      <c r="G24" s="33" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="14" t="inlineStr">
@@ -868,11 +971,15 @@
           <t>4. Build Evidence</t>
         </is>
       </c>
+      <c r="C25" s="33" t="n"/>
       <c r="D25" s="15" t="inlineStr">
         <is>
           <t>9 features — commit hashes, repos, key files, functions</t>
         </is>
       </c>
+      <c r="E25" s="34" t="n"/>
+      <c r="F25" s="34" t="n"/>
+      <c r="G25" s="33" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="14" t="inlineStr">
@@ -880,11 +987,15 @@
           <t>5. Discussion Log</t>
         </is>
       </c>
+      <c r="C26" s="33" t="n"/>
       <c r="D26" s="15" t="inlineStr">
         <is>
           <t>Team Q&amp;A — decisions, owners, due dates</t>
         </is>
       </c>
+      <c r="E26" s="34" t="n"/>
+      <c r="F26" s="34" t="n"/>
+      <c r="G26" s="33" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="B27" s="14" t="inlineStr">
@@ -892,11 +1003,15 @@
           <t>6. Sprint Plan</t>
         </is>
       </c>
+      <c r="C27" s="33" t="n"/>
       <c r="D27" s="15" t="inlineStr">
         <is>
           <t>Sprint 0–7 — scope, velocity, status, notes</t>
         </is>
       </c>
+      <c r="E27" s="34" t="n"/>
+      <c r="F27" s="34" t="n"/>
+      <c r="G27" s="33" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="31">
@@ -908,8 +1023,8 @@
     <mergeCell ref="D25:G25"/>
     <mergeCell ref="D24:G24"/>
     <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B27:C27"/>
     <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B27:C27"/>
     <mergeCell ref="F7:G7"/>
     <mergeCell ref="D23:G23"/>
     <mergeCell ref="D26:G26"/>
@@ -943,7 +1058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:P33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1074,7 +1189,7 @@
       </c>
       <c r="F2" s="21" t="inlineStr">
         <is>
-          <t>POC — not merged to org</t>
+          <t>Done — V3 in org repo (Temperature /weather/analyze-wind) + windApi.ts + WindResultsPanel</t>
         </is>
       </c>
       <c r="G2" s="18" t="inlineStr">
@@ -1092,7 +1207,7 @@
       </c>
       <c r="J2" s="19" t="inlineStr">
         <is>
-          <t>Vishwas721/sat (sat04/)</t>
+          <t>SiteAnalysisToolV3/backend/Temperature/ + frontend/src/services/</t>
         </is>
       </c>
       <c r="K2" s="18" t="inlineStr">
@@ -1117,12 +1232,12 @@
       </c>
       <c r="O2" s="18" t="inlineStr">
         <is>
-          <t>FVD-09</t>
+          <t>FVD-09 / FVD-17</t>
         </is>
       </c>
       <c r="P2" s="19" t="inlineStr">
         <is>
-          <t>POC in personal repo. Must merge to org before integration.</t>
+          <t>V3 production backend supersedes POC. Open-Meteo ERA5 daily.</t>
         </is>
       </c>
     </row>
@@ -1144,12 +1259,12 @@
       </c>
       <c r="D3" s="22" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>SAT-8</t>
         </is>
       </c>
       <c r="E3" s="24" t="inlineStr">
         <is>
-          <t>No ticket</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F3" s="25" t="inlineStr">
@@ -1234,7 +1349,7 @@
       </c>
       <c r="F4" s="20" t="inlineStr">
         <is>
-          <t>Done — local backend</t>
+          <t>Done — V3 in org repo (backend/Temperature/, port 8000)</t>
         </is>
       </c>
       <c r="G4" s="18" t="inlineStr">
@@ -1252,12 +1367,12 @@
       </c>
       <c r="J4" s="19" t="inlineStr">
         <is>
-          <t>Site-Analysis-Tool/src/Backend/Temperature/</t>
+          <t>SiteAnalysisToolV3/backend/Temperature/</t>
         </is>
       </c>
       <c r="K4" s="18" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>4bf53de</t>
         </is>
       </c>
       <c r="L4" s="18" t="inlineStr">
@@ -1282,7 +1397,7 @@
       </c>
       <c r="P4" s="19" t="inlineStr">
         <is>
-          <t>First candidate for integration. Backend fully tested.</t>
+          <t>V3 integrated.</t>
         </is>
       </c>
     </row>
@@ -1304,12 +1419,12 @@
       </c>
       <c r="D5" s="22" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>SAT-11</t>
         </is>
       </c>
       <c r="E5" s="24" t="inlineStr">
         <is>
-          <t>No ticket</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F5" s="20" t="inlineStr">
@@ -1394,7 +1509,7 @@
       </c>
       <c r="F6" s="20" t="inlineStr">
         <is>
-          <t>Done — local backend</t>
+          <t>Done — V3 in org repo (backend/SunPath/, port 8001, shadow engine enhanced)</t>
         </is>
       </c>
       <c r="G6" s="18" t="inlineStr">
@@ -1412,12 +1527,12 @@
       </c>
       <c r="J6" s="19" t="inlineStr">
         <is>
-          <t>Sprint0_User_Stories + Site-Analysis-Tool/src/Backend/SunPath/</t>
+          <t>SiteAnalysisToolV3/backend/SunPath/</t>
         </is>
       </c>
       <c r="K6" s="18" t="inlineStr">
         <is>
-          <t>944c5b8</t>
+          <t>4bf53de</t>
         </is>
       </c>
       <c r="L6" s="18" t="inlineStr">
@@ -1442,7 +1557,7 @@
       </c>
       <c r="P6" s="19" t="inlineStr">
         <is>
-          <t>Backend done. Shadow casting and solstice export not implemented.</t>
+          <t>V3: shadow engine, face-shadow engine, OSM extractor added.</t>
         </is>
       </c>
     </row>
@@ -1464,17 +1579,17 @@
       </c>
       <c r="D7" s="22" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>SAT-66 / SAT-207</t>
         </is>
       </c>
       <c r="E7" s="24" t="inlineStr">
         <is>
-          <t>No ticket</t>
+          <t>Backlog / To Do</t>
         </is>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>No code</t>
+          <t>Done — V3 in org repo (SiteAnalysisToolV3/backend/Terrain/)</t>
         </is>
       </c>
       <c r="G7" s="22" t="inlineStr">
@@ -1492,12 +1607,12 @@
       </c>
       <c r="J7" s="23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Site-Analysis/SiteAnalysisToolV3 — backend/Terrain/</t>
         </is>
       </c>
       <c r="K7" s="22" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>4bf53de</t>
         </is>
       </c>
       <c r="L7" s="22" t="inlineStr">
@@ -1522,7 +1637,7 @@
       </c>
       <c r="P7" s="23" t="inlineStr">
         <is>
-          <t>MERIT DEM already used in flood service — slope calc is a natural extension.</t>
+          <t>SAT-66 (Backlog) and SAT-207 (To Do) — duplicate stories. Implemented in V3 Terrain backend. See FVD-10.</t>
         </is>
       </c>
     </row>
@@ -1634,7 +1749,7 @@
       </c>
       <c r="F9" s="20" t="inlineStr">
         <is>
-          <t>Done — local backend</t>
+          <t>Done — V3 in org repo (backend/FloodPlains/, port 8002)</t>
         </is>
       </c>
       <c r="G9" s="22" t="inlineStr">
@@ -1652,12 +1767,12 @@
       </c>
       <c r="J9" s="23" t="inlineStr">
         <is>
-          <t>SiteAnalysis_GEE + Site-Analysis-Tool/src/Backend/FloodPlains/</t>
+          <t>SiteAnalysisToolV3/backend/FloodPlains/</t>
         </is>
       </c>
       <c r="K9" s="22" t="inlineStr">
         <is>
-          <t>edd4c29</t>
+          <t>4bf53de</t>
         </is>
       </c>
       <c r="L9" s="22" t="inlineStr">
@@ -1682,7 +1797,7 @@
       </c>
       <c r="P9" s="23" t="inlineStr">
         <is>
-          <t>4-component scoring done. Historical flood event data not integrated.</t>
+          <t>V3 integrated. GEE chart + PDF + map renderer added.</t>
         </is>
       </c>
     </row>
@@ -2358,7 +2473,7 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>No code</t>
+          <t>Done — V3 in org repo (SiteAnalysisToolV3/frontend/src/lib/energy-carbon.ts)</t>
         </is>
       </c>
       <c r="G18" s="18" t="inlineStr">
@@ -2374,12 +2489,12 @@
       </c>
       <c r="J18" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Site-Analysis/SiteAnalysisToolV3 — frontend/src/lib/</t>
         </is>
       </c>
       <c r="K18" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>4bf53de</t>
         </is>
       </c>
       <c r="L18" s="18" t="inlineStr">
@@ -3029,6 +3144,566 @@
       <c r="P26" s="19" t="inlineStr">
         <is>
           <t>No external data source identified. Likely curated static dataset by region.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>US-05</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Terrain Analysis (Slope/Aspect/Buildable Zones)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>SAT-66 / SAT-207</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Backlog / To Do</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Done — V3 in org repo (SiteAnalysisToolV3/backend/Terrain/)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>V3 team</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>8</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Must Have</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Site-Analysis/SiteAnalysisToolV3 — backend/Terrain/</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>4bf53de</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>services/terrain/</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>feature.terrain.analysis</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>FVD-10</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>New Terrain backend port 8003. Slope/aspect/buildable/hazard/suitability. SAT-66 (Backlog) + SAT-207 (To Do) are duplicate stories — need resolution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>US-NEW-01</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>3D Simulation Engine (Three.js + OSM context)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>SAT-218</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Done — V3 in org repo (SiteAnalysisToolV3/frontend/src/simulation/)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>V3 team</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>21</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Must Have</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Site-Analysis/SiteAnalysisToolV3 — frontend/src/simulation/</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>dc4288a</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>apps/web/simulation/</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>N/A (frontend)</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>feature.simulation.3d</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>FVD-11</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>SceneCanvas 5317 lines. Three.js + R3F. Terrain DEM, OSM context, proposal buildings, sketch detail. SAT-219/220/221 subtasks all To Do — FVD-11 docs cover them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>US-09</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>NBC 2016 Constraints + Generative Design Engine</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>No ticket</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Done — V3 in org repo (SiteAnalysisToolV3/frontend/src/lib/)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>V3 team</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>13</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Must Have</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Site-Analysis/SiteAnalysisToolV3 — frontend/src/lib/</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>4bf53de</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>apps/web/lib/</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>N/A (frontend)</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>feature.regulatory.nbc</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>FVD-12</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>FAR/setbacks/coverage/parking from NBC 2016. 6 typology presets. AI enhancer scoring. NBC data accuracy unverified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>US-10</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Energy Use &amp; Embodied Carbon (ECBC 2017)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>No ticket</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Done — V3 in org repo (SiteAnalysisToolV3/frontend/src/lib/energy-carbon.ts)</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>V3 team</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>8</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Must Have</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Site-Analysis/SiteAnalysisToolV3 — frontend/src/lib/</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>4bf53de</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>apps/web/lib/</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>N/A (frontend)</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>feature.regulatory.ecbc</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>FVD-13</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>ECBC 2017 baseline EUI × 5 climate zones. Live carbon in simulation. Embodied carbon LCA deferred.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>US-NEW-02</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Pedestrian Wind + Noise + Thermal Comfort (Client-Side)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>No ticket</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Done — V3 in org repo (SiteAnalysisToolV3/frontend/src/lib/)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>V3 team</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>13</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Should Have</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Site-Analysis/SiteAnalysisToolV3 — frontend/src/lib/</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>4bf53de</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>apps/web/lib/</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>N/A (frontend)</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>feature.simulation.microclimate</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>FVD-14</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>wind-sim.ts (CFD approx, Lawson criteria), noise-sim.ts (CPCB), thermal-comfort.ts (ISO 7730 PMV). No UI panels yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>US-NEW-03</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>BIM/CAD Exports (PDF + IFC + GLTF)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>No ticket</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Done — V3 in org repo (SiteAnalysisToolV3/frontend/src/lib/)</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>V3 team</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>8</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Should Have</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Site-Analysis/SiteAnalysisToolV3 — frontend/src/lib/</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>4bf53de</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>apps/web/lib/</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>N/A (frontend)</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>feature.export.bim</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>FVD-15</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>jsPDF A4 report, web-ifc IFC2x3, Three.js GLTFExporter GLB. IFC coordinates are x=0,z=0 placeholders. No export UI found in V3 frontend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>US-NEW-04</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Realtime Collaboration &amp; Project Sharing</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>No ticket</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Service done — in org repo (SiteAnalysisToolV3/frontend/src/services/)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>V3 team</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>13</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Should Have</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Site-Analysis/SiteAnalysisToolV3 — frontend/src/services/</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>4bf53de</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>apps/web/services/</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>N/A (frontend)</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>feature.collaboration.realtime</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>FVD-16</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Supabase realtime presence + invites + share tokens. Services built but SimulationRoot has no save/share UI yet. isReadOnly flag not enforced in SceneCanvas.</t>
         </is>
       </c>
     </row>
@@ -3917,7 +4592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3994,10 +4669,14 @@
       </c>
       <c r="F2" s="24" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="G2" s="19" t="inlineStr"/>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="G2" s="19" t="inlineStr">
+        <is>
+          <t>V3 full implementation in Site-Analysis/SiteAnalysisToolV3 (commit 685547b). FVD-17 documents V3 wind analysis. FVD-09 POC deprecated.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="22" t="inlineStr">
@@ -4060,10 +4739,14 @@
       </c>
       <c r="F4" s="24" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="G4" s="19" t="inlineStr"/>
+          <t>Partially Resolved</t>
+        </is>
+      </c>
+      <c r="G4" s="19" t="inlineStr">
+        <is>
+          <t>SAT-8 exists (In Progress). Still no code found in V3. Needs implementation.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="22" t="inlineStr">
@@ -4192,10 +4875,14 @@
       </c>
       <c r="F8" s="24" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="G8" s="19" t="inlineStr"/>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="G8" s="19" t="inlineStr">
+        <is>
+          <t>Feature Registry updated: US-01 (Wind) = Done, US-02 (Temperature) = Done. V3 in org repo confirmed.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="22" t="inlineStr">
@@ -4559,6 +5246,393 @@
         </is>
       </c>
       <c r="G19" s="23" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Terrain Analysis (US-05)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>No Org Push</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>backend/Terrain/ exists only in local SiteAnalysisToolV3. Must push to Site-Analysis org before Sprint 3 integration.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>V3 team</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>3D Simulation (US-NEW-01)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Not Wired to Analysis APIs</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Simulation AnalysisPanel uses local proposal metrics only — does not call SunPath/Flood/Temperature backends. Wind/solar context absent.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>V3 team</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Phase 2 integration work item</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>3D Simulation (US-NEW-01)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Persistence Not Wired</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>simulationProjectService.ts + collaborationService.ts exist but SimulationRoot has no save/share UI. Projects cannot be saved from simulation flow.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>V3 team</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>3D Simulation (US-NEW-01)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>CSG Booleans Approximated</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>csg-ops.ts (three-bvh-csg) exists but not wired. Union/subtract/intersect use bounding-box approximation.</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>V3 team</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>NBC Engine (US-09)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Data Accuracy Unverified</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>FAR/setback lookup tables in modeling-math.ts not independently verified against NBC 2016 Table 15 by a licensed architect.</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>V3 team</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Architecture review needed before prod use</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Wind/Noise/Thermal (US-NEW-02)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>No UI Panels</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>wind-sim.ts, noise-sim.ts, thermal-comfort.ts are complete libraries but no frontend panels expose them to users.</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>V3 team</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>UI component work needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>IFC Export (US-NEW-03)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Coordinates Are Placeholders</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>export-ifc.ts uses x=0, z=0 for all buildings ("In a full implementation, convert lat/lng to meters"). IFC not usable in Revit until fixed.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>V3 team</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>All V3 Features (FVD-10–17)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>No Jira Tickets</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>8 new features in SiteAnalysisToolV3 have no Jira tickets, no sprint assignment, no story points confirmed.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Chirag</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Raise stories before Sprint 4 planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Rainfall Analysis (US-03)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Code Unverified</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>SAT-11 exists (In Progress). Karthik claims Done but code not located in any scanned repo. Commit 9a548ef referenced in V3 git log but files not explored yet.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Karthik</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Check SiteAnalysisToolV3 commit 9a548ef. Explore frontend/src/lib/rainfall* or similar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>BIM Export IFC (US-NEW-03)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Incomplete Feature</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>export-ifc.ts: createBuildingMesh() uses x=0,z=0 placeholders. Comment says "In a full implementation, convert lat/lng to meters". IFC files unusable in BIM tools until fixed.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>V3 team</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Implement Haversine lat/lng→XZ offset in createBuildingMesh(). Site origin = project centroid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Simulation Libraries (FVD-12/13/14/15)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>No UI Wiring</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>NBC generative engine, ECBC energy calc, wind/noise/thermal comfort, and BIM exports have no UI panels in V3 SimulationRoot. Libraries complete but not accessible to users.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>V3 team</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Build: SimulationToolbar with export button, NBCPanel, EnergyPanel, WindComfortPanel, NoiseMappingPanel. Wire to existing store actions.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
@@ -4573,7 +5647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4952,6 +6026,302 @@
       <c r="G10" s="19" t="inlineStr">
         <is>
           <t>GET /analysis/wind/climatology, fetch_gee_wind_data(), build_rose(), get_imd_season(), get_orientation_advice()</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Terrain Analysis Backend V3</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SiteAnalysisToolV3/backend/Terrain/</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>app/main.py, app/terrain_utils.py, app/models.py</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>POST /analyze/terrain, POST /analyze/terrain/polygon, POST /profile, POST /inspect</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Wind Analysis V3 (Production)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>SiteAnalysisToolV3/backend/Temperature/</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>SAT-4</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>app/routers/weather.py, frontend/src/services/windApi.ts</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>GET /weather/analyze-wind → WindAnalysis{rose[16], monthly[12], seasonal[4], summary.crossVentDir}</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>3D Simulation Engine</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>SiteAnalysisToolV3/frontend/src/simulation/</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>app/SimulationRoot.tsx, components/scene/SceneCanvas.tsx (5317 lines), utils/terrain-dem.ts, lib/osm-fetch.ts</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Terrain DEM (Mapbox RGB), OSM context (Overpass), Three.js scene, Sketch detail editor</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>NBC + Generative Engine</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>SiteAnalysisToolV3/frontend/src/lib/</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>lib/nbc-constraints.ts, lib/modeling-math.ts, lib/generative-engine.ts, lib/ai-enhancer.ts</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>calculateNBCConstraints(), generateVariants(), scoreVariant() — 5 India climate zones × 6 typologies</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Energy &amp; Carbon (ECBC 2017)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>SiteAnalysisToolV3/frontend/src/lib/</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>lib/energy-carbon.ts</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>calculateBuildingEUI(), calculateTotalEnergyUse() — ECBC 2017 baselines × 5 climate zones</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Wind/Noise/PMV Simulations</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>SiteAnalysisToolV3/frontend/src/lib/</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>lib/wind-sim.ts, lib/noise-sim.ts, lib/thermal-comfort.ts</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>calculateWindComfortGrid() (Lawson), calculateNoiseGrid() (CPCB), calculatePMV() (ISO 7730)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BIM/CAD Exports</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>SiteAnalysisToolV3/frontend/src/lib/</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>lib/export-pdf.ts (jsPDF), lib/export-ifc.ts (web-ifc), lib/export-gltf.ts (Three.js GLTFExporter)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>generateProjectReport() → PDF Blob, exportBuildingsToIFC() → IFC2x3 Blob, exportBuildingsToGLTF() → GLB Blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Realtime Collaboration Services</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>SiteAnalysisToolV3/frontend/src/services/</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>services/collaborationService.ts, services/realtimeService.ts, services/simulationProjectService.ts, hooks/useCollaborationStore.ts</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>inviteCollaborator(), broadcastModelChange(), saveSimulationProject() — Supabase Realtime + Presence</t>
         </is>
       </c>
     </row>
@@ -5511,7 +6881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5880,6 +7250,46 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sprint 4 (planned)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>55</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Push V3 backends to org (Terrain, Temperature/Wind, SunPath V3, FloodPlains V3). Wire simulation to analysis APIs. Add export UI. Raise Jira stories for FVD-10 to FVD-17.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>V3 validation complete 2026-05-26. 8 new FVDs written (FVD-10–17). Primary gaps: no org push, no Jira tickets, simulation not wired to APIs.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>